<commit_message>
Included doc in the app for user and AI
</commit_message>
<xml_diff>
--- a/profiles/comptoirs-oceaniques/data.xlsx
+++ b/profiles/comptoirs-oceaniques/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Rapports\Version 072026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\DEV\Report-Generator\profiles\comptoirs-oceaniques\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A2E82E-79BD-4F13-B7EC-5819DE31C2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3C7F198-21F3-4140-A5D1-E76068344BCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -19,11 +19,27 @@
     <sheet name="espece-critere_qualite" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1377" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="418">
   <si>
     <t>nom rapport generé</t>
   </si>
@@ -1304,6 +1320,9 @@
   </si>
   <si>
     <t>NOVOCIB Rapport d'essai 261016-13.docx</t>
+  </si>
+  <si>
+    <t>thon obèse</t>
   </si>
 </sst>
 </file>
@@ -2011,7 +2030,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
+    <cellStyle name="Pourcentage" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2290,7 +2309,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AF65"/>
-  <sheetFormatPr defaultColWidth="20.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="20.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" customWidth="1"/>
@@ -7879,8 +7898,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33.28515625" customWidth="1"/>
     <col min="2" max="2" width="19.28515625" customWidth="1"/>
@@ -8004,6 +8023,14 @@
       </c>
       <c r="B15" t="s">
         <v>363</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>151</v>
+      </c>
+      <c r="B16" t="s">
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -8015,7 +8042,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.85546875" customWidth="1"/>
     <col min="2" max="2" width="21.5703125" customWidth="1"/>
@@ -8229,7 +8256,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.140625" customWidth="1"/>
     <col min="2" max="2" width="42.85546875" customWidth="1"/>

</xml_diff>